<commit_message>
cambios en el frontend
</commit_message>
<xml_diff>
--- a/BACKEND/uploads/archivo_subido.xlsx
+++ b/BACKEND/uploads/archivo_subido.xlsx
@@ -1,26 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29029"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="21929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sena\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\yacardenas\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A05ABD33-4005-4A49-A7CA-7C7022D02329}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F5F6877F-DA2E-4F04-8443-CCCDFC5B02BD}" xr6:coauthVersionLast="44" xr6:coauthVersionMax="44" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Datos" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="26">
   <si>
     <t>TIPO DE DOCUMENTO</t>
   </si>
@@ -43,52 +43,61 @@
     <t>CC</t>
   </si>
   <si>
-    <t>YAIR</t>
-  </si>
-  <si>
-    <t>MAYO</t>
-  </si>
-  <si>
-    <t>TI</t>
-  </si>
-  <si>
-    <t>ejemplo tipo</t>
-  </si>
-  <si>
-    <t>JUNIO</t>
-  </si>
-  <si>
-    <t>YAIR MAL</t>
-  </si>
-  <si>
-    <t>FALLECIDO</t>
-  </si>
-  <si>
-    <t>FEBRERO</t>
-  </si>
-  <si>
-    <t>PPT</t>
-  </si>
-  <si>
-    <t>MARZO</t>
-  </si>
-  <si>
-    <t>JOSE URBANO PARRA GUZMAN</t>
-  </si>
-  <si>
-    <t>SEPTIEMBRE</t>
-  </si>
-  <si>
-    <t>CE</t>
-  </si>
-  <si>
-    <t>OCTUBRE</t>
-  </si>
-  <si>
-    <t>ANTONIO  CASTAÑEDA</t>
-  </si>
-  <si>
-    <t>ARNULFO  BRIÑEZ QUESADA</t>
+    <t>1005826381</t>
+  </si>
+  <si>
+    <t>N/A</t>
+  </si>
+  <si>
+    <t>9</t>
+  </si>
+  <si>
+    <t>Septiembre</t>
+  </si>
+  <si>
+    <t>2020</t>
+  </si>
+  <si>
+    <t>1106452473</t>
+  </si>
+  <si>
+    <t>12</t>
+  </si>
+  <si>
+    <t>Julio</t>
+  </si>
+  <si>
+    <t>2005</t>
+  </si>
+  <si>
+    <t>1106452858</t>
+  </si>
+  <si>
+    <t>2006</t>
+  </si>
+  <si>
+    <t>1109297711</t>
+  </si>
+  <si>
+    <t>10</t>
+  </si>
+  <si>
+    <t>Marzo</t>
+  </si>
+  <si>
+    <t>2011</t>
+  </si>
+  <si>
+    <t>1193519425</t>
+  </si>
+  <si>
+    <t>11</t>
+  </si>
+  <si>
+    <t>Junio</t>
+  </si>
+  <si>
+    <t>2019</t>
   </si>
 </sst>
 </file>
@@ -144,12 +153,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -452,14 +460,8 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F10"/>
+  <dimension ref="A1:F6"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="27" customWidth="1"/>
-    <col min="2" max="2" width="29" customWidth="1"/>
-    <col min="3" max="3" width="40" customWidth="1"/>
-    <col min="4" max="6" width="13" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
@@ -485,199 +487,103 @@
       <c r="A2" t="s">
         <v>6</v>
       </c>
-      <c r="B2">
-        <v>1108453116</v>
+      <c r="B2" t="s">
+        <v>7</v>
       </c>
       <c r="C2" t="s">
-        <v>7</v>
-      </c>
-      <c r="D2">
-        <v>28</v>
+        <v>8</v>
+      </c>
+      <c r="D2" t="s">
+        <v>9</v>
       </c>
       <c r="E2" t="s">
-        <v>8</v>
-      </c>
-      <c r="F2">
-        <v>2024</v>
+        <v>10</v>
+      </c>
+      <c r="F2" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>9</v>
-      </c>
-      <c r="B3">
-        <v>1108453116</v>
+        <v>6</v>
+      </c>
+      <c r="B3" t="s">
+        <v>12</v>
       </c>
       <c r="C3" t="s">
-        <v>10</v>
-      </c>
-      <c r="D3">
-        <v>28</v>
+        <v>8</v>
+      </c>
+      <c r="D3" t="s">
+        <v>13</v>
       </c>
       <c r="E3" t="s">
-        <v>11</v>
-      </c>
-      <c r="F3">
-        <v>2024</v>
+        <v>14</v>
+      </c>
+      <c r="F3" t="s">
+        <v>15</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>6</v>
       </c>
-      <c r="B4">
-        <v>1108453116</v>
+      <c r="B4" t="s">
+        <v>16</v>
       </c>
       <c r="C4" t="s">
-        <v>12</v>
-      </c>
-      <c r="D4">
-        <v>29</v>
+        <v>8</v>
+      </c>
+      <c r="D4" t="s">
+        <v>13</v>
       </c>
       <c r="E4" t="s">
-        <v>11</v>
-      </c>
-      <c r="F4">
-        <v>2024</v>
+        <v>10</v>
+      </c>
+      <c r="F4" t="s">
+        <v>17</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>6</v>
       </c>
-      <c r="B5">
-        <v>21202856</v>
+      <c r="B5" t="s">
+        <v>18</v>
       </c>
       <c r="C5" t="s">
-        <v>13</v>
-      </c>
-      <c r="D5">
+        <v>8</v>
+      </c>
+      <c r="D5" t="s">
+        <v>19</v>
+      </c>
+      <c r="E5" t="s">
         <v>20</v>
       </c>
-      <c r="E5" t="s">
-        <v>14</v>
-      </c>
-      <c r="F5">
-        <v>1985</v>
+      <c r="F5" t="s">
+        <v>21</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>15</v>
-      </c>
-      <c r="B6">
-        <v>1108453116</v>
+        <v>6</v>
+      </c>
+      <c r="B6" t="s">
+        <v>22</v>
       </c>
       <c r="C6" t="s">
-        <v>10</v>
-      </c>
-      <c r="D6">
-        <v>20</v>
+        <v>8</v>
+      </c>
+      <c r="D6" t="s">
+        <v>23</v>
       </c>
       <c r="E6" t="s">
-        <v>16</v>
-      </c>
-      <c r="F6">
-        <v>1985</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>6</v>
-      </c>
-      <c r="B7">
-        <v>5814634</v>
-      </c>
-      <c r="C7" t="s">
-        <v>17</v>
-      </c>
-      <c r="D7">
-        <v>10</v>
-      </c>
-      <c r="E7" t="s">
-        <v>18</v>
-      </c>
-      <c r="F7">
-        <v>1962</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>19</v>
-      </c>
-      <c r="B8">
-        <v>1108453116</v>
-      </c>
-      <c r="C8" t="s">
-        <v>10</v>
-      </c>
-      <c r="D8">
-        <v>10</v>
-      </c>
-      <c r="E8" t="s">
-        <v>20</v>
-      </c>
-      <c r="F8">
-        <v>1962</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>6</v>
-      </c>
-      <c r="B9" s="2">
-        <v>5817677</v>
-      </c>
-      <c r="C9" t="s">
-        <v>21</v>
-      </c>
-      <c r="D9">
-        <v>4</v>
-      </c>
-      <c r="E9" t="s">
-        <v>16</v>
-      </c>
-      <c r="F9">
-        <v>1964</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
-        <v>6</v>
-      </c>
-      <c r="B10" s="2">
-        <v>5999992</v>
-      </c>
-      <c r="C10" t="s">
-        <v>22</v>
-      </c>
-      <c r="D10">
-        <v>8</v>
-      </c>
-      <c r="E10" t="s">
-        <v>20</v>
-      </c>
-      <c r="F10">
-        <v>1971</v>
+        <v>24</v>
+      </c>
+      <c r="F6" t="s">
+        <v>25</v>
       </c>
     </row>
   </sheetData>
-  <dataValidations count="4">
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Entrada inválida" error="Debe seleccionar uno de los valores válidos: CC, TI, CE, PPT" promptTitle="Tipo de Documento" prompt="Seleccione un tipo de documento válido: CC, TI, CE, PPT" sqref="A2:A1000" xr:uid="{00000000-0002-0000-0000-000000000000}">
-      <formula1>"CC,TI,CE,PPT"</formula1>
-    </dataValidation>
-    <dataValidation type="whole" allowBlank="1" showErrorMessage="1" errorTitle="Día inválido" error="El día debe ser un número entre 1 y 31" promptTitle="Día" prompt="Ingrese un día válido (1-31)" sqref="D2:D1000" xr:uid="{00000000-0002-0000-0000-000001000000}">
-      <formula1>1</formula1>
-      <formula2>31</formula2>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Mes inválido" error="Debe seleccionar un mes válido en mayúsculas" promptTitle="Mes" prompt="Seleccione un mes válido" sqref="E2:E1000" xr:uid="{00000000-0002-0000-0000-000002000000}">
-      <formula1>"ENERO,FEBRERO,MARZO,ABRIL,MAYO,JUNIO,JULIO,AGOSTO,SEPTIEMBRE,OCTUBRE,NOVIEMBRE,DICIEMBRE"</formula1>
-    </dataValidation>
-    <dataValidation type="whole" allowBlank="1" showErrorMessage="1" errorTitle="Año inválido" error="El año debe estar entre 1900 y 2025 (no se permiten años futuros)" promptTitle="Año" prompt="Ingrese un año válido (1900-2025)" sqref="F2:F1000" xr:uid="{00000000-0002-0000-0000-000003000000}">
-      <formula1>1900</formula1>
-      <formula2>2025</formula2>
-    </dataValidation>
-  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
avances en el frontend
</commit_message>
<xml_diff>
--- a/BACKEND/uploads/archivo_subido.xlsx
+++ b/BACKEND/uploads/archivo_subido.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="21929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28526"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\yacardenas\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\yacardenas\Downloads\05 AGOSTO_pruebass\3207631_\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F5F6877F-DA2E-4F04-8443-CCCDFC5B02BD}" xr6:coauthVersionLast="44" xr6:coauthVersionMax="44" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{75FBEEC3-C757-4401-BC82-6EA4AA9262E3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="36">
   <si>
     <t>TIPO DE DOCUMENTO</t>
   </si>
@@ -43,61 +43,91 @@
     <t>CC</t>
   </si>
   <si>
-    <t>1005826381</t>
+    <t>1005827023</t>
   </si>
   <si>
     <t>N/A</t>
   </si>
   <si>
-    <t>9</t>
+    <t>27</t>
   </si>
   <si>
     <t>Septiembre</t>
   </si>
   <si>
+    <t>2019</t>
+  </si>
+  <si>
+    <t>1005827457</t>
+  </si>
+  <si>
+    <t>25</t>
+  </si>
+  <si>
+    <t>Julio</t>
+  </si>
+  <si>
     <t>2020</t>
   </si>
   <si>
-    <t>1106452473</t>
-  </si>
-  <si>
-    <t>12</t>
-  </si>
-  <si>
-    <t>Julio</t>
-  </si>
-  <si>
-    <t>2005</t>
-  </si>
-  <si>
-    <t>1106452858</t>
+    <t>1005827593</t>
+  </si>
+  <si>
+    <t>19</t>
+  </si>
+  <si>
+    <t>Junio</t>
+  </si>
+  <si>
+    <t>1012447841</t>
+  </si>
+  <si>
+    <t>1</t>
+  </si>
+  <si>
+    <t>Diciembre</t>
+  </si>
+  <si>
+    <t>2015</t>
+  </si>
+  <si>
+    <t>1023865072</t>
+  </si>
+  <si>
+    <t>14</t>
+  </si>
+  <si>
+    <t>2004</t>
+  </si>
+  <si>
+    <t>1097392739</t>
+  </si>
+  <si>
+    <t>28</t>
+  </si>
+  <si>
+    <t>Noviembre</t>
   </si>
   <si>
     <t>2006</t>
   </si>
   <si>
-    <t>1109297711</t>
-  </si>
-  <si>
-    <t>10</t>
+    <t>1106484570</t>
+  </si>
+  <si>
+    <t>5</t>
   </si>
   <si>
     <t>Marzo</t>
   </si>
   <si>
-    <t>2011</t>
-  </si>
-  <si>
-    <t>1193519425</t>
-  </si>
-  <si>
-    <t>11</t>
-  </si>
-  <si>
-    <t>Junio</t>
-  </si>
-  <si>
-    <t>2019</t>
+    <t>2009</t>
+  </si>
+  <si>
+    <t>1106484719</t>
+  </si>
+  <si>
+    <t>23</t>
   </si>
 </sst>
 </file>
@@ -460,7 +490,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F6"/>
+  <dimension ref="A1:F9"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -534,13 +564,13 @@
         <v>8</v>
       </c>
       <c r="D4" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="E4" t="s">
-        <v>10</v>
+        <v>18</v>
       </c>
       <c r="F4" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
@@ -548,19 +578,19 @@
         <v>6</v>
       </c>
       <c r="B5" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C5" t="s">
         <v>8</v>
       </c>
       <c r="D5" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="E5" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="F5" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
@@ -568,19 +598,79 @@
         <v>6</v>
       </c>
       <c r="B6" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C6" t="s">
         <v>8</v>
       </c>
       <c r="D6" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E6" t="s">
-        <v>24</v>
+        <v>10</v>
       </c>
       <c r="F6" t="s">
         <v>25</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>6</v>
+      </c>
+      <c r="B7" t="s">
+        <v>26</v>
+      </c>
+      <c r="C7" t="s">
+        <v>8</v>
+      </c>
+      <c r="D7" t="s">
+        <v>27</v>
+      </c>
+      <c r="E7" t="s">
+        <v>28</v>
+      </c>
+      <c r="F7" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>6</v>
+      </c>
+      <c r="B8" t="s">
+        <v>30</v>
+      </c>
+      <c r="C8" t="s">
+        <v>8</v>
+      </c>
+      <c r="D8" t="s">
+        <v>31</v>
+      </c>
+      <c r="E8" t="s">
+        <v>32</v>
+      </c>
+      <c r="F8" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>6</v>
+      </c>
+      <c r="B9" t="s">
+        <v>34</v>
+      </c>
+      <c r="C9" t="s">
+        <v>8</v>
+      </c>
+      <c r="D9" t="s">
+        <v>35</v>
+      </c>
+      <c r="E9" t="s">
+        <v>14</v>
+      </c>
+      <c r="F9" t="s">
+        <v>33</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
cambio de nombre de archivos en backend
</commit_message>
<xml_diff>
--- a/BACKEND/uploads/archivo_subido.xlsx
+++ b/BACKEND/uploads/archivo_subido.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F25"/>
+  <dimension ref="A1:F30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -479,17 +479,17 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>1003752366</t>
+          <t>1006093296</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>ERIKA SIRLEY CASTAÑEDA CRUZ</t>
+          <t>MAICOL STIVEN FALLA LEYTON</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>24</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -499,7 +499,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>2018</t>
+          <t>2020</t>
         </is>
       </c>
     </row>
@@ -511,27 +511,27 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>1003752386</t>
+          <t>1006149386</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>LEONIDAS CASTAÑEDA AMAYA</t>
+          <t>JOSE NEDER ALAPE CASTILLO</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>21</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>AGOSTO</t>
+          <t>FEBRERO</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>2021</t>
+          <t>2017</t>
         </is>
       </c>
     </row>
@@ -543,12 +543,12 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>1071629289</t>
+          <t>1007248274</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>LEIDY KATHERINE QUEVEDO ROMERO</t>
+          <t>YENIFER TIQUE BOCANEGRA</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -558,12 +558,12 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>OCTUBRE</t>
+          <t>NOVIEMBRE</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>2007</t>
+          <t>2014</t>
         </is>
       </c>
     </row>
@@ -575,27 +575,27 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>1121832842</t>
+          <t>1007326248</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>GLORIA STELLA CAMPO MEDINA</t>
+          <t>LUIS ROBERTO BOCANEGRA BARRETO</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>31</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>JULIO</t>
+          <t>AGOSTO</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>2005</t>
+          <t>2011</t>
         </is>
       </c>
     </row>
@@ -607,27 +607,27 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>11297947</t>
+          <t>1007710504</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>FERNANDO REY PEÑALOZA</t>
+          <t>MELIZA PEDRAZA ALAPE</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>13</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>SEPTIEMBRE</t>
+          <t>DICIEMBRE</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>1975</t>
+          <t>2018</t>
         </is>
       </c>
     </row>
@@ -639,27 +639,27 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>17335022</t>
+          <t>1007787228</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>JAIME MAHECHA MEDINA</t>
+          <t>NATALIA PRIETO CUMACO</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>5</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>MAYO</t>
+          <t>NOVIEMBRE</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>1985</t>
+          <t>2015</t>
         </is>
       </c>
     </row>
@@ -671,27 +671,27 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>20611169</t>
+          <t>1020749191</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>MARIA FLORENCIA MORALES DE AMAYA</t>
+          <t>DIANA ALEJANDRA GIRALDO CORTES</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>JULIO</t>
+          <t>FEBRERO</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>1969</t>
+          <t>2008</t>
         </is>
       </c>
     </row>
@@ -703,27 +703,27 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>20634423</t>
+          <t>1105684798</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>LUZ STELLA MARTINEZ MORENO</t>
+          <t>JUAN CAMILO LOZANO HERNANDEZ</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>19</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>SEPTIEMBRE</t>
+          <t>JULIO</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>1988</t>
+          <t>2011</t>
         </is>
       </c>
     </row>
@@ -735,12 +735,12 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>20816304</t>
+          <t>1106394251</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>ANA YOLANDA BELTRAN VELASQUEZ</t>
+          <t>MARISELA BARRIOS CRUZ</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -750,12 +750,12 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>SEPTIEMBRE</t>
+          <t>JULIO</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>1985</t>
+          <t>2006</t>
         </is>
       </c>
     </row>
@@ -767,27 +767,27 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>28786631</t>
+          <t>1110173966</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>FLOR ALBA PARRA</t>
+          <t>LILIANA TIMOTE TAPIERO</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>2</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>JULIO</t>
+          <t>FEBRERO</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>1977</t>
+          <t>2006</t>
         </is>
       </c>
     </row>
@@ -799,27 +799,27 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>28787644</t>
+          <t>1110174203</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>MARIA CELMIRA DAZA LOPEZ</t>
+          <t>SORLEY PRIETO CUMACO</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>29</t>
+          <t>28</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>SEPTIEMBRE</t>
+          <t>JUNIO</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>1983</t>
+          <t>2006</t>
         </is>
       </c>
     </row>
@@ -831,27 +831,27 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>28788525</t>
+          <t>1110175251</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>MARIA NELSY JIMENEZ RODRIGUEZ</t>
+          <t>MARIA VICTORIA DIAZ ARIAS</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>22</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>MARZO</t>
+          <t>NOVIEMBRE</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>1992</t>
+          <t>2007</t>
         </is>
       </c>
     </row>
@@ -863,12 +863,12 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>28788815</t>
+          <t>1110176770</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>MARIA NUBIA SAAVEDRA PRADA</t>
+          <t>JAIME ELVER MENDOZA ALAPE</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -878,12 +878,12 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>SEPTIEMBRE</t>
+          <t>MAYO</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>1995</t>
+          <t>2010</t>
         </is>
       </c>
     </row>
@@ -895,27 +895,27 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>28788947</t>
+          <t>1110459909</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>LUZ HERMINDA CRUZ DIAZ</t>
+          <t>MARIA CAMILA ASCENCIO MACIAS</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>25</t>
+          <t>9</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>JUNIO</t>
+          <t>MAYO</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>1997</t>
+          <t>2023</t>
         </is>
       </c>
     </row>
@@ -927,27 +927,27 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>28789111</t>
+          <t>1110487036</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>AURORA MACIAS FONSECA</t>
+          <t>YIDY NEREY PIÑERES RAMIREZ</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>2</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>MAYO</t>
+          <t>AGOSTO</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>1999</t>
+          <t>2007</t>
         </is>
       </c>
     </row>
@@ -959,27 +959,27 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>3014782</t>
+          <t>1192794186</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>JOSE EUGENIO MALDONADO PINILLA</t>
+          <t>FLOR ANGELICA GUTIERREZ DUCUARA</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>12</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>AGOSTO</t>
+          <t>MARZO</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>1972</t>
+          <t>2015</t>
         </is>
       </c>
     </row>
@@ -991,17 +991,17 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>40277641</t>
+          <t>1193529089</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>ESMERALDA ZABALA VALDERRAMA</t>
+          <t>ANGIE JULIANA ALAPE TAPIERO</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>28</t>
+          <t>23</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -1011,7 +1011,7 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>1996</t>
+          <t>2016</t>
         </is>
       </c>
     </row>
@@ -1023,27 +1023,27 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>40361451</t>
+          <t>14106485</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>LUZ ELBA CASTRO RIVERA</t>
+          <t>YOAN MANUEL SALDAÑA ANGARITA</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>11</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>AGOSTO</t>
+          <t>DICIEMBRE</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>1991</t>
+          <t>1997</t>
         </is>
       </c>
     </row>
@@ -1055,27 +1055,27 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>51553749</t>
+          <t>28866884</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>STELLA RAIRAN CRUZ</t>
+          <t>ADELINA TAPIERO TAPIERO</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>17</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>DICIEMBRE</t>
+          <t>SEPTIEMBRE</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>1978</t>
+          <t>1990</t>
         </is>
       </c>
     </row>
@@ -1087,27 +1087,27 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>52050248</t>
+          <t>28868392</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>LUZ NOELIA PERDOMO MUNERA</t>
+          <t>ANAYANCI PRIETO BRIÑEZ</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>22</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>JUNIO</t>
+          <t>MAYO</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>1990</t>
+          <t>1996</t>
         </is>
       </c>
     </row>
@@ -1119,27 +1119,27 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>5933442</t>
+          <t>28868619</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>FIDELIGNO AVILA RAMIREZ</t>
+          <t>ERIKA DARLENI HERRAN</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>18</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>DICIEMBRE</t>
+          <t>MARZO</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>1975</t>
+          <t>1997</t>
         </is>
       </c>
     </row>
@@ -1151,27 +1151,27 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>5935181</t>
+          <t>28869696</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>FREDY EDUARDO AMAYA MORALES</t>
+          <t>MAGDA YURANY COLLAZOS SALDAÑA</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>29</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>DICIEMBRE</t>
+          <t>JUNIO</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>1985</t>
+          <t>2000</t>
         </is>
       </c>
     </row>
@@ -1183,57 +1183,217 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>6030427</t>
+          <t>30347439</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>HERNANDO MUÑOZ ROMERO</t>
+          <t>NANCY LOZANO TORRES</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>12</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>NOVIEMBRE</t>
+          <t>FEBRERO</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>1984</t>
+          <t>1987</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
+          <t>CC</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>65753363</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>LUZ ELIDA CAMACHO RIAÑO</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>JULIO</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>1990</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>CC</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>79751537</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>WILLIAM JOEL MORENO MONTENEGRO</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>JULIO</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>1992</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>CC</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>93020553</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>NORBEY MENDOZA ALAPE</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>23</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>ABRIL</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>1999</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>CC</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>93020639</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>RUBEN DARIO MATOMA JOANIAS</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>AGOSTO</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>1999</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>CC</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>93414016</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>ALFONSO OLAYA GALARZA</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>NOVIEMBRE</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>1997</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
           <t>TI</t>
         </is>
       </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>1106363625</t>
-        </is>
-      </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>AMAYA MACIAS ZHARICK DAYANA</t>
-        </is>
-      </c>
-      <c r="D25" t="inlineStr">
-        <is>
-          <t>03</t>
-        </is>
-      </c>
-      <c r="E25" t="inlineStr">
-        <is>
-          <t>JUNIO</t>
-        </is>
-      </c>
-      <c r="F25" t="inlineStr">
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>1030284516</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>TOVAR VILLALBA MARIA PAZ</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>OCTUBRE</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
         <is>
           <t>2010</t>
         </is>

</xml_diff>

<commit_message>
Segunda opcion de ppt
</commit_message>
<xml_diff>
--- a/BACKEND/uploads/archivo_subido.xlsx
+++ b/BACKEND/uploads/archivo_subido.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\yacardenas\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7362FE0F-EB76-4DAD-BC65-18DAB3758714}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{74437ECB-3D91-454F-8C01-B8B0E40E1333}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1080" yWindow="1080" windowWidth="13230" windowHeight="7950" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
   <si>
     <t>TIPO DE DOCUMENTO</t>
   </si>
@@ -47,6 +47,15 @@
   </si>
   <si>
     <t>MAYO</t>
+  </si>
+  <si>
+    <t>PPT</t>
+  </si>
+  <si>
+    <t>veneco</t>
+  </si>
+  <si>
+    <t>FEBRERO</t>
   </si>
 </sst>
 </file>
@@ -409,7 +418,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:F3"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="27" customWidth="1"/>
@@ -456,6 +465,26 @@
       </c>
       <c r="F2">
         <v>2024</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>9</v>
+      </c>
+      <c r="B3">
+        <v>122</v>
+      </c>
+      <c r="C3" t="s">
+        <v>10</v>
+      </c>
+      <c r="D3">
+        <v>23</v>
+      </c>
+      <c r="E3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F3">
+        <v>2021</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Reintenta con las filas cuando se cae la pagina
</commit_message>
<xml_diff>
--- a/BACKEND/uploads/archivo_subido.xlsx
+++ b/BACKEND/uploads/archivo_subido.xlsx
@@ -5,22 +5,22 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\yacardenas\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\yacardenas\Desktop\21 DE OCTUBRE_PRUEBA CERTIGRANJA\3324483\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C403579D-353F-4FC5-8ABB-B0452287AA26}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{869220C2-7B63-415B-96B3-83872F30A586}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Datos" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="37">
   <si>
     <t>TIPO DE DOCUMENTO</t>
   </si>
@@ -43,16 +43,94 @@
     <t>CC</t>
   </si>
   <si>
-    <t>n/A</t>
+    <t>1003805788</t>
+  </si>
+  <si>
+    <t>OSWALDO GRACIA POLO</t>
+  </si>
+  <si>
+    <t>18</t>
+  </si>
+  <si>
+    <t>NOVIEMBRE</t>
+  </si>
+  <si>
+    <t>2019</t>
+  </si>
+  <si>
+    <t>ENERO</t>
+  </si>
+  <si>
+    <t>JUNIO</t>
+  </si>
+  <si>
+    <t>2011</t>
+  </si>
+  <si>
+    <t>DICIEMBRE</t>
+  </si>
+  <si>
+    <t>1110505697</t>
+  </si>
+  <si>
+    <t>NATALI BARRERO LEAL</t>
+  </si>
+  <si>
+    <t>7</t>
+  </si>
+  <si>
+    <t>2009</t>
+  </si>
+  <si>
+    <t>1111122386</t>
+  </si>
+  <si>
+    <t>JUAN JOSE SOTO PALMA</t>
+  </si>
+  <si>
+    <t>2</t>
+  </si>
+  <si>
+    <t>2022</t>
+  </si>
+  <si>
+    <t>1113664721</t>
+  </si>
+  <si>
+    <t>INGRI YULEYSI RIVAS VARELA</t>
+  </si>
+  <si>
+    <t>15</t>
+  </si>
+  <si>
+    <t>14207214</t>
+  </si>
+  <si>
+    <t>JAIRO EULOGIO MORALES</t>
+  </si>
+  <si>
+    <t>30</t>
+  </si>
+  <si>
+    <t>ABRIL</t>
+  </si>
+  <si>
+    <t>1971</t>
+  </si>
+  <si>
+    <t>TI</t>
+  </si>
+  <si>
+    <t>YAIR ALEXANDER CARDENAS GUZMAN</t>
+  </si>
+  <si>
+    <t>31</t>
   </si>
   <si>
     <t>MAYO</t>
   </si>
   <si>
-    <t>TI</t>
-  </si>
-  <si>
-    <t>JUNIO</t>
+    <t>PPT</t>
   </si>
 </sst>
 </file>
@@ -117,7 +195,7 @@
   <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -421,13 +499,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:F8"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="27" customWidth="1"/>
-    <col min="2" max="2" width="29" customWidth="1"/>
+    <col min="1" max="2" width="20" customWidth="1"/>
     <col min="3" max="3" width="40" customWidth="1"/>
-    <col min="4" max="6" width="13" customWidth="1"/>
+    <col min="4" max="4" width="10" customWidth="1"/>
+    <col min="5" max="5" width="15" customWidth="1"/>
+    <col min="6" max="6" width="10" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -454,56 +533,156 @@
       <c r="A2" t="s">
         <v>6</v>
       </c>
-      <c r="B2">
-        <v>1108453116</v>
+      <c r="B2" t="s">
+        <v>7</v>
       </c>
       <c r="C2" t="s">
-        <v>7</v>
-      </c>
-      <c r="D2">
-        <v>28</v>
+        <v>8</v>
+      </c>
+      <c r="D2" t="s">
+        <v>9</v>
       </c>
       <c r="E2" t="s">
-        <v>8</v>
-      </c>
-      <c r="F2">
-        <v>2024</v>
+        <v>15</v>
+      </c>
+      <c r="F2" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>9</v>
-      </c>
-      <c r="B3">
+        <v>6</v>
+      </c>
+      <c r="B3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C3" t="s">
+        <v>17</v>
+      </c>
+      <c r="D3" t="s">
+        <v>18</v>
+      </c>
+      <c r="E3" t="s">
+        <v>12</v>
+      </c>
+      <c r="F3" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>6</v>
+      </c>
+      <c r="B4" t="s">
+        <v>20</v>
+      </c>
+      <c r="C4" t="s">
+        <v>21</v>
+      </c>
+      <c r="D4" t="s">
+        <v>22</v>
+      </c>
+      <c r="E4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F4" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>6</v>
+      </c>
+      <c r="B5" t="s">
+        <v>24</v>
+      </c>
+      <c r="C5" t="s">
+        <v>25</v>
+      </c>
+      <c r="D5" t="s">
+        <v>26</v>
+      </c>
+      <c r="E5" t="s">
+        <v>10</v>
+      </c>
+      <c r="F5" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>6</v>
+      </c>
+      <c r="B6" t="s">
+        <v>27</v>
+      </c>
+      <c r="C6" t="s">
+        <v>28</v>
+      </c>
+      <c r="D6" t="s">
+        <v>29</v>
+      </c>
+      <c r="E6" t="s">
+        <v>30</v>
+      </c>
+      <c r="F6" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>32</v>
+      </c>
+      <c r="B7">
         <v>1108453116</v>
       </c>
-      <c r="C3" t="s">
-        <v>7</v>
-      </c>
-      <c r="D3">
-        <v>28</v>
-      </c>
-      <c r="E3" t="s">
-        <v>10</v>
-      </c>
-      <c r="F3">
-        <v>2024</v>
+      <c r="C7" t="s">
+        <v>33</v>
+      </c>
+      <c r="D7" t="s">
+        <v>34</v>
+      </c>
+      <c r="E7" t="s">
+        <v>35</v>
+      </c>
+      <c r="F7">
+        <v>2000</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>36</v>
+      </c>
+      <c r="B8">
+        <v>1108453116</v>
+      </c>
+      <c r="C8" t="s">
+        <v>33</v>
+      </c>
+      <c r="D8">
+        <v>1</v>
+      </c>
+      <c r="E8" t="s">
+        <v>13</v>
+      </c>
+      <c r="F8">
+        <v>2000</v>
       </c>
     </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
   <dataValidations count="4">
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Entrada inválida" error="Debe seleccionar uno de los valores válidos: CC, TI, CE, PPT" promptTitle="Tipo de Documento" prompt="Seleccione un tipo de documento válido: CC, TI, CE, PPT" sqref="A2:A1000" xr:uid="{00000000-0002-0000-0000-000000000000}">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Entrada inválida" error="Debe seleccionar uno de los valores válidos: CC, TI, CE, PPT" promptTitle="Tipo de Documento" prompt="Seleccione un tipo de documento válido: CC, TI, CE, PPT" sqref="A2:A978" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>"CC,TI,CE,PPT"</formula1>
     </dataValidation>
-    <dataValidation type="whole" allowBlank="1" showErrorMessage="1" errorTitle="Día inválido" error="El día debe ser un número entre 1 y 31" promptTitle="Día" prompt="Ingrese un día válido (1-31)" sqref="D2:D1000" xr:uid="{00000000-0002-0000-0000-000001000000}">
+    <dataValidation type="whole" allowBlank="1" showErrorMessage="1" errorTitle="Día inválido" error="El día debe ser un número entre 1 y 31" promptTitle="Día" prompt="Ingrese un día válido (1-31)" sqref="D2:D978" xr:uid="{00000000-0002-0000-0000-000001000000}">
       <formula1>1</formula1>
       <formula2>31</formula2>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Mes inválido" error="Debe seleccionar un mes válido en mayúsculas" promptTitle="Mes" prompt="Seleccione un mes válido" sqref="E2:E1000" xr:uid="{00000000-0002-0000-0000-000002000000}">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Mes inválido" error="Debe seleccionar un mes válido en mayúsculas" promptTitle="Mes" prompt="Seleccione un mes válido" sqref="E2:E978" xr:uid="{00000000-0002-0000-0000-000002000000}">
       <formula1>"ENERO,FEBRERO,MARZO,ABRIL,MAYO,JUNIO,JULIO,AGOSTO,SEPTIEMBRE,OCTUBRE,NOVIEMBRE,DICIEMBRE"</formula1>
     </dataValidation>
-    <dataValidation type="whole" allowBlank="1" showErrorMessage="1" errorTitle="Año inválido" error="El año debe estar entre 1900 y 2025 (no se permiten años futuros)" promptTitle="Año" prompt="Ingrese un año válido (1900-2025)" sqref="F2:F1000" xr:uid="{00000000-0002-0000-0000-000003000000}">
+    <dataValidation type="whole" allowBlank="1" showErrorMessage="1" errorTitle="Año inválido" error="El año debe estar entre 1900 y 2025" promptTitle="Año" prompt="Ingrese un año válido (1900-2025)" sqref="F2:F978" xr:uid="{00000000-0002-0000-0000-000003000000}">
       <formula1>1900</formula1>
       <formula2>2025</formula2>
     </dataValidation>

</xml_diff>